<commit_message>
v2 - browser audit, console logging, screenshots, improved dashboard
</commit_message>
<xml_diff>
--- a/data/sites.xlsx
+++ b/data/sites.xlsx
@@ -9,6 +9,7 @@
   <sheets>
     <sheet name="sites" sheetId="1" state="visible" r:id="rId1"/>
     <sheet name="endpoints" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet name="exceptions" sheetId="3" state="visible" r:id="rId3"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -633,7 +634,7 @@
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>https://httpbin.org/status/200</t>
+          <t>https://httpbin.org/status/503</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
@@ -664,6 +665,88 @@
       </c>
       <c r="E7" t="n">
         <v>2000</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:G2"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="inlineStr">
+        <is>
+          <t>rule_id</t>
+        </is>
+      </c>
+      <c r="B1" t="inlineStr">
+        <is>
+          <t>enabled</t>
+        </is>
+      </c>
+      <c r="C1" t="inlineStr">
+        <is>
+          <t>site_id</t>
+        </is>
+      </c>
+      <c r="D1" t="inlineStr">
+        <is>
+          <t>endpoint_id</t>
+        </is>
+      </c>
+      <c r="E1" t="inlineStr">
+        <is>
+          <t>match_type</t>
+        </is>
+      </c>
+      <c r="F1" t="inlineStr">
+        <is>
+          <t>pattern</t>
+        </is>
+      </c>
+      <c r="G1" t="inlineStr">
+        <is>
+          <t>notes</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>GH_WEBGL_1</t>
+        </is>
+      </c>
+      <c r="B2" t="n">
+        <v>1</v>
+      </c>
+      <c r="C2" t="n">
+        <v>3</v>
+      </c>
+      <c r="D2" t="n">
+        <v>3</v>
+      </c>
+      <c r="E2" t="inlineStr">
+        <is>
+          <t>contains</t>
+        </is>
+      </c>
+      <c r="F2" t="inlineStr">
+        <is>
+          <t>GPU stall due to ReadPixels</t>
+        </is>
+      </c>
+      <c r="G2" t="inlineStr">
+        <is>
+          <t>Ignore GitHub WebGL GPU stall warning for testing</t>
+        </is>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
v3 - switch to real data, reset monitoring data, status handling updates, frontend refresh
</commit_message>
<xml_diff>
--- a/data/sites.xlsx
+++ b/data/sites.xlsx
@@ -415,7 +415,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C6"/>
+  <dimension ref="A1:C43"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -441,7 +441,7 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>Google</t>
+          <t>416-flowers.com</t>
         </is>
       </c>
       <c r="C2" t="n">
@@ -454,7 +454,7 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>Wikipedia</t>
+          <t>a3cf.org</t>
         </is>
       </c>
       <c r="C3" t="n">
@@ -467,7 +467,7 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>GitHub</t>
+          <t>lejardin.com</t>
         </is>
       </c>
       <c r="C4" t="n">
@@ -480,7 +480,7 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>Httpbin503</t>
+          <t>albertgelman.com</t>
         </is>
       </c>
       <c r="C5" t="n">
@@ -493,10 +493,491 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>Httpbin200</t>
+          <t>arellicleaning.com</t>
         </is>
       </c>
       <c r="C6" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="n">
+        <v>6</v>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>argocustoms.com</t>
+        </is>
+      </c>
+      <c r="C7" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="n">
+        <v>7</v>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>askhoward.com</t>
+        </is>
+      </c>
+      <c r="C8" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="n">
+        <v>8</v>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>boxshop.ca</t>
+        </is>
+      </c>
+      <c r="C9" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="n">
+        <v>9</v>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>canadianimportexport.ca</t>
+        </is>
+      </c>
+      <c r="C10" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="n">
+        <v>10</v>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>commercialcleaninggta.com</t>
+        </is>
+      </c>
+      <c r="C11" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="n">
+        <v>11</v>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>cozycomfortplus.com</t>
+        </is>
+      </c>
+      <c r="C12" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="n">
+        <v>12</v>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>elginmillsendodontic.com</t>
+        </is>
+      </c>
+      <c r="C13" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="n">
+        <v>13</v>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>endodonticsondonmills.com</t>
+        </is>
+      </c>
+      <c r="C14" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="n">
+        <v>14</v>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>goldenrescue.ca</t>
+        </is>
+      </c>
+      <c r="C15" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="n">
+        <v>15</v>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>helpinghandsdoula.com</t>
+        </is>
+      </c>
+      <c r="C16" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="n">
+        <v>16</v>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>iamyoga.ca</t>
+        </is>
+      </c>
+      <c r="C17" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="n">
+        <v>17</v>
+      </c>
+      <c r="B18" t="inlineStr">
+        <is>
+          <t>iconbedbugs.ca</t>
+        </is>
+      </c>
+      <c r="C18" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="n">
+        <v>18</v>
+      </c>
+      <c r="B19" t="inlineStr">
+        <is>
+          <t>iconbird.ca</t>
+        </is>
+      </c>
+      <c r="C19" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="n">
+        <v>19</v>
+      </c>
+      <c r="B20" t="inlineStr">
+        <is>
+          <t>iconpest.ca</t>
+        </is>
+      </c>
+      <c r="C20" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="n">
+        <v>20</v>
+      </c>
+      <c r="B21" t="inlineStr">
+        <is>
+          <t>identos.com</t>
+        </is>
+      </c>
+      <c r="C21" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="n">
+        <v>21</v>
+      </c>
+      <c r="B22" t="inlineStr">
+        <is>
+          <t>iranda.ca</t>
+        </is>
+      </c>
+      <c r="C22" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="n">
+        <v>22</v>
+      </c>
+      <c r="B23" t="inlineStr">
+        <is>
+          <t>marketing-dentist.com</t>
+        </is>
+      </c>
+      <c r="C23" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="n">
+        <v>23</v>
+      </c>
+      <c r="B24" t="inlineStr">
+        <is>
+          <t>metrobit.ca</t>
+        </is>
+      </c>
+      <c r="C24" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="n">
+        <v>24</v>
+      </c>
+      <c r="B25" t="inlineStr">
+        <is>
+          <t>nuday.com</t>
+        </is>
+      </c>
+      <c r="C25" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="n">
+        <v>25</v>
+      </c>
+      <c r="B26" t="inlineStr">
+        <is>
+          <t>officecleaningbrampton.com</t>
+        </is>
+      </c>
+      <c r="C26" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="n">
+        <v>26</v>
+      </c>
+      <c r="B27" t="inlineStr">
+        <is>
+          <t>officecleaninggta.com</t>
+        </is>
+      </c>
+      <c r="C27" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" t="n">
+        <v>27</v>
+      </c>
+      <c r="B28" t="inlineStr">
+        <is>
+          <t>officecleaningvaughan.com</t>
+        </is>
+      </c>
+      <c r="C28" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" t="n">
+        <v>28</v>
+      </c>
+      <c r="B29" t="inlineStr">
+        <is>
+          <t>packyourboxes.com</t>
+        </is>
+      </c>
+      <c r="C29" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" t="n">
+        <v>29</v>
+      </c>
+      <c r="B30" t="inlineStr">
+        <is>
+          <t>pante-a.com</t>
+        </is>
+      </c>
+      <c r="C30" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" t="n">
+        <v>30</v>
+      </c>
+      <c r="B31" t="inlineStr">
+        <is>
+          <t>profuneralflowers.com</t>
+        </is>
+      </c>
+      <c r="C31" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" t="n">
+        <v>31</v>
+      </c>
+      <c r="B32" t="inlineStr">
+        <is>
+          <t>redsealvending.ca</t>
+        </is>
+      </c>
+      <c r="C32" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" t="n">
+        <v>32</v>
+      </c>
+      <c r="B33" t="inlineStr">
+        <is>
+          <t>surgearrest.com</t>
+        </is>
+      </c>
+      <c r="C33" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" t="n">
+        <v>33</v>
+      </c>
+      <c r="B34" t="inlineStr">
+        <is>
+          <t>toplinedesign.ca</t>
+        </is>
+      </c>
+      <c r="C34" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" t="n">
+        <v>34</v>
+      </c>
+      <c r="B35" t="inlineStr">
+        <is>
+          <t>wildlifecontrol.ca</t>
+        </is>
+      </c>
+      <c r="C35" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" t="n">
+        <v>35</v>
+      </c>
+      <c r="B36" t="inlineStr">
+        <is>
+          <t>zigma.ca</t>
+        </is>
+      </c>
+      <c r="C36" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" t="n">
+        <v>36</v>
+      </c>
+      <c r="B37" t="inlineStr">
+        <is>
+          <t>zigship.com</t>
+        </is>
+      </c>
+      <c r="C37" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" t="n">
+        <v>37</v>
+      </c>
+      <c r="B38" t="inlineStr">
+        <is>
+          <t>oneworldimmigration.ca</t>
+        </is>
+      </c>
+      <c r="C38" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" t="n">
+        <v>38</v>
+      </c>
+      <c r="B39" t="inlineStr">
+        <is>
+          <t>airconditioner-furnace.ca</t>
+        </is>
+      </c>
+      <c r="C39" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" t="n">
+        <v>39</v>
+      </c>
+      <c r="B40" t="inlineStr">
+        <is>
+          <t>bed-bugs-treatments.com</t>
+        </is>
+      </c>
+      <c r="C40" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" t="n">
+        <v>40</v>
+      </c>
+      <c r="B41" t="inlineStr">
+        <is>
+          <t>sultanxpress.ca</t>
+        </is>
+      </c>
+      <c r="C41" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" t="n">
+        <v>41</v>
+      </c>
+      <c r="B42" t="inlineStr">
+        <is>
+          <t>wildlifepro.ca</t>
+        </is>
+      </c>
+      <c r="C42" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" t="n">
+        <v>42</v>
+      </c>
+      <c r="B43" t="inlineStr">
+        <is>
+          <t>reboundproducts.com</t>
+        </is>
+      </c>
+      <c r="C43" t="n">
         <v>1</v>
       </c>
     </row>
@@ -511,7 +992,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E7"/>
+  <dimension ref="A1:E43"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -550,7 +1031,7 @@
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>https://www.google.com</t>
+          <t>https://416-flowers.com</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
@@ -571,7 +1052,7 @@
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>https://www.wikipedia.org</t>
+          <t>https://a3cf.org</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
@@ -592,7 +1073,7 @@
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>https://github.com/</t>
+          <t>https://lejardin.com</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
@@ -613,7 +1094,7 @@
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>https://httpbin.org/status/503</t>
+          <t>https://albertgelman.com</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
@@ -634,7 +1115,7 @@
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>https://httpbin.org/status/503</t>
+          <t>https://arellicleaning.com</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
@@ -651,11 +1132,11 @@
         <v>6</v>
       </c>
       <c r="B7" t="n">
-        <v>1</v>
+        <v>6</v>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>http://google.com</t>
+          <t>https://argocustoms.com</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
@@ -664,6 +1145,762 @@
         </is>
       </c>
       <c r="E7" t="n">
+        <v>2000</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="n">
+        <v>7</v>
+      </c>
+      <c r="B8" t="n">
+        <v>7</v>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>https://askhoward.com</t>
+        </is>
+      </c>
+      <c r="D8" t="inlineStr">
+        <is>
+          <t>GET</t>
+        </is>
+      </c>
+      <c r="E8" t="n">
+        <v>2000</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="n">
+        <v>8</v>
+      </c>
+      <c r="B9" t="n">
+        <v>8</v>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>https://boxshop.ca</t>
+        </is>
+      </c>
+      <c r="D9" t="inlineStr">
+        <is>
+          <t>GET</t>
+        </is>
+      </c>
+      <c r="E9" t="n">
+        <v>2000</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="n">
+        <v>9</v>
+      </c>
+      <c r="B10" t="n">
+        <v>9</v>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>https://canadianimportexport.ca</t>
+        </is>
+      </c>
+      <c r="D10" t="inlineStr">
+        <is>
+          <t>GET</t>
+        </is>
+      </c>
+      <c r="E10" t="n">
+        <v>2000</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="n">
+        <v>10</v>
+      </c>
+      <c r="B11" t="n">
+        <v>10</v>
+      </c>
+      <c r="C11" t="inlineStr">
+        <is>
+          <t>https://commercialcleaninggta.com</t>
+        </is>
+      </c>
+      <c r="D11" t="inlineStr">
+        <is>
+          <t>GET</t>
+        </is>
+      </c>
+      <c r="E11" t="n">
+        <v>2000</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="n">
+        <v>11</v>
+      </c>
+      <c r="B12" t="n">
+        <v>11</v>
+      </c>
+      <c r="C12" t="inlineStr">
+        <is>
+          <t>https://cozycomfortplus.com</t>
+        </is>
+      </c>
+      <c r="D12" t="inlineStr">
+        <is>
+          <t>GET</t>
+        </is>
+      </c>
+      <c r="E12" t="n">
+        <v>2000</v>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="n">
+        <v>12</v>
+      </c>
+      <c r="B13" t="n">
+        <v>12</v>
+      </c>
+      <c r="C13" t="inlineStr">
+        <is>
+          <t>https://elginmillsendodontic.com</t>
+        </is>
+      </c>
+      <c r="D13" t="inlineStr">
+        <is>
+          <t>GET</t>
+        </is>
+      </c>
+      <c r="E13" t="n">
+        <v>2000</v>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="n">
+        <v>13</v>
+      </c>
+      <c r="B14" t="n">
+        <v>13</v>
+      </c>
+      <c r="C14" t="inlineStr">
+        <is>
+          <t>https://endodonticsondonmills.com</t>
+        </is>
+      </c>
+      <c r="D14" t="inlineStr">
+        <is>
+          <t>GET</t>
+        </is>
+      </c>
+      <c r="E14" t="n">
+        <v>2000</v>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="n">
+        <v>14</v>
+      </c>
+      <c r="B15" t="n">
+        <v>14</v>
+      </c>
+      <c r="C15" t="inlineStr">
+        <is>
+          <t>https://goldenrescue.ca</t>
+        </is>
+      </c>
+      <c r="D15" t="inlineStr">
+        <is>
+          <t>GET</t>
+        </is>
+      </c>
+      <c r="E15" t="n">
+        <v>2000</v>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="n">
+        <v>15</v>
+      </c>
+      <c r="B16" t="n">
+        <v>15</v>
+      </c>
+      <c r="C16" t="inlineStr">
+        <is>
+          <t>https://helpinghandsdoula.com</t>
+        </is>
+      </c>
+      <c r="D16" t="inlineStr">
+        <is>
+          <t>GET</t>
+        </is>
+      </c>
+      <c r="E16" t="n">
+        <v>2000</v>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="n">
+        <v>16</v>
+      </c>
+      <c r="B17" t="n">
+        <v>16</v>
+      </c>
+      <c r="C17" t="inlineStr">
+        <is>
+          <t>https://iamyoga.ca</t>
+        </is>
+      </c>
+      <c r="D17" t="inlineStr">
+        <is>
+          <t>GET</t>
+        </is>
+      </c>
+      <c r="E17" t="n">
+        <v>2000</v>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="n">
+        <v>17</v>
+      </c>
+      <c r="B18" t="n">
+        <v>17</v>
+      </c>
+      <c r="C18" t="inlineStr">
+        <is>
+          <t>https://iconbedbugs.ca</t>
+        </is>
+      </c>
+      <c r="D18" t="inlineStr">
+        <is>
+          <t>GET</t>
+        </is>
+      </c>
+      <c r="E18" t="n">
+        <v>2000</v>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="n">
+        <v>18</v>
+      </c>
+      <c r="B19" t="n">
+        <v>18</v>
+      </c>
+      <c r="C19" t="inlineStr">
+        <is>
+          <t>https://iconbird.ca</t>
+        </is>
+      </c>
+      <c r="D19" t="inlineStr">
+        <is>
+          <t>GET</t>
+        </is>
+      </c>
+      <c r="E19" t="n">
+        <v>2000</v>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="n">
+        <v>19</v>
+      </c>
+      <c r="B20" t="n">
+        <v>19</v>
+      </c>
+      <c r="C20" t="inlineStr">
+        <is>
+          <t>https://iconpest.ca</t>
+        </is>
+      </c>
+      <c r="D20" t="inlineStr">
+        <is>
+          <t>GET</t>
+        </is>
+      </c>
+      <c r="E20" t="n">
+        <v>2000</v>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="n">
+        <v>20</v>
+      </c>
+      <c r="B21" t="n">
+        <v>20</v>
+      </c>
+      <c r="C21" t="inlineStr">
+        <is>
+          <t>https://identos.com</t>
+        </is>
+      </c>
+      <c r="D21" t="inlineStr">
+        <is>
+          <t>GET</t>
+        </is>
+      </c>
+      <c r="E21" t="n">
+        <v>2000</v>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="n">
+        <v>21</v>
+      </c>
+      <c r="B22" t="n">
+        <v>21</v>
+      </c>
+      <c r="C22" t="inlineStr">
+        <is>
+          <t>https://iranda.ca</t>
+        </is>
+      </c>
+      <c r="D22" t="inlineStr">
+        <is>
+          <t>GET</t>
+        </is>
+      </c>
+      <c r="E22" t="n">
+        <v>2000</v>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="n">
+        <v>22</v>
+      </c>
+      <c r="B23" t="n">
+        <v>22</v>
+      </c>
+      <c r="C23" t="inlineStr">
+        <is>
+          <t>https://marketing-dentist.com</t>
+        </is>
+      </c>
+      <c r="D23" t="inlineStr">
+        <is>
+          <t>GET</t>
+        </is>
+      </c>
+      <c r="E23" t="n">
+        <v>2000</v>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="n">
+        <v>23</v>
+      </c>
+      <c r="B24" t="n">
+        <v>23</v>
+      </c>
+      <c r="C24" t="inlineStr">
+        <is>
+          <t>https://metrobit.ca</t>
+        </is>
+      </c>
+      <c r="D24" t="inlineStr">
+        <is>
+          <t>GET</t>
+        </is>
+      </c>
+      <c r="E24" t="n">
+        <v>2000</v>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="n">
+        <v>24</v>
+      </c>
+      <c r="B25" t="n">
+        <v>24</v>
+      </c>
+      <c r="C25" t="inlineStr">
+        <is>
+          <t>https://nuday.com</t>
+        </is>
+      </c>
+      <c r="D25" t="inlineStr">
+        <is>
+          <t>GET</t>
+        </is>
+      </c>
+      <c r="E25" t="n">
+        <v>2000</v>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="n">
+        <v>25</v>
+      </c>
+      <c r="B26" t="n">
+        <v>25</v>
+      </c>
+      <c r="C26" t="inlineStr">
+        <is>
+          <t>https://officecleaningbrampton.com</t>
+        </is>
+      </c>
+      <c r="D26" t="inlineStr">
+        <is>
+          <t>GET</t>
+        </is>
+      </c>
+      <c r="E26" t="n">
+        <v>2000</v>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="n">
+        <v>26</v>
+      </c>
+      <c r="B27" t="n">
+        <v>26</v>
+      </c>
+      <c r="C27" t="inlineStr">
+        <is>
+          <t>https://officecleaninggta.com</t>
+        </is>
+      </c>
+      <c r="D27" t="inlineStr">
+        <is>
+          <t>GET</t>
+        </is>
+      </c>
+      <c r="E27" t="n">
+        <v>2000</v>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" t="n">
+        <v>27</v>
+      </c>
+      <c r="B28" t="n">
+        <v>27</v>
+      </c>
+      <c r="C28" t="inlineStr">
+        <is>
+          <t>https://officecleaningvaughan.com</t>
+        </is>
+      </c>
+      <c r="D28" t="inlineStr">
+        <is>
+          <t>GET</t>
+        </is>
+      </c>
+      <c r="E28" t="n">
+        <v>2000</v>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" t="n">
+        <v>28</v>
+      </c>
+      <c r="B29" t="n">
+        <v>28</v>
+      </c>
+      <c r="C29" t="inlineStr">
+        <is>
+          <t>https://packyourboxes.com</t>
+        </is>
+      </c>
+      <c r="D29" t="inlineStr">
+        <is>
+          <t>GET</t>
+        </is>
+      </c>
+      <c r="E29" t="n">
+        <v>2000</v>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" t="n">
+        <v>29</v>
+      </c>
+      <c r="B30" t="n">
+        <v>29</v>
+      </c>
+      <c r="C30" t="inlineStr">
+        <is>
+          <t>https://pante-a.com</t>
+        </is>
+      </c>
+      <c r="D30" t="inlineStr">
+        <is>
+          <t>GET</t>
+        </is>
+      </c>
+      <c r="E30" t="n">
+        <v>2000</v>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" t="n">
+        <v>30</v>
+      </c>
+      <c r="B31" t="n">
+        <v>30</v>
+      </c>
+      <c r="C31" t="inlineStr">
+        <is>
+          <t>https://profuneralflowers.com</t>
+        </is>
+      </c>
+      <c r="D31" t="inlineStr">
+        <is>
+          <t>GET</t>
+        </is>
+      </c>
+      <c r="E31" t="n">
+        <v>2000</v>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" t="n">
+        <v>31</v>
+      </c>
+      <c r="B32" t="n">
+        <v>31</v>
+      </c>
+      <c r="C32" t="inlineStr">
+        <is>
+          <t>https://redsealvending.ca</t>
+        </is>
+      </c>
+      <c r="D32" t="inlineStr">
+        <is>
+          <t>GET</t>
+        </is>
+      </c>
+      <c r="E32" t="n">
+        <v>2000</v>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" t="n">
+        <v>32</v>
+      </c>
+      <c r="B33" t="n">
+        <v>32</v>
+      </c>
+      <c r="C33" t="inlineStr">
+        <is>
+          <t>https://surgearrest.com</t>
+        </is>
+      </c>
+      <c r="D33" t="inlineStr">
+        <is>
+          <t>GET</t>
+        </is>
+      </c>
+      <c r="E33" t="n">
+        <v>2000</v>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" t="n">
+        <v>33</v>
+      </c>
+      <c r="B34" t="n">
+        <v>33</v>
+      </c>
+      <c r="C34" t="inlineStr">
+        <is>
+          <t>https://toplinedesign.ca</t>
+        </is>
+      </c>
+      <c r="D34" t="inlineStr">
+        <is>
+          <t>GET</t>
+        </is>
+      </c>
+      <c r="E34" t="n">
+        <v>2000</v>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" t="n">
+        <v>34</v>
+      </c>
+      <c r="B35" t="n">
+        <v>34</v>
+      </c>
+      <c r="C35" t="inlineStr">
+        <is>
+          <t>https://wildlifecontrol.ca</t>
+        </is>
+      </c>
+      <c r="D35" t="inlineStr">
+        <is>
+          <t>GET</t>
+        </is>
+      </c>
+      <c r="E35" t="n">
+        <v>2000</v>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" t="n">
+        <v>35</v>
+      </c>
+      <c r="B36" t="n">
+        <v>35</v>
+      </c>
+      <c r="C36" t="inlineStr">
+        <is>
+          <t>https://zigma.ca</t>
+        </is>
+      </c>
+      <c r="D36" t="inlineStr">
+        <is>
+          <t>GET</t>
+        </is>
+      </c>
+      <c r="E36" t="n">
+        <v>2000</v>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" t="n">
+        <v>36</v>
+      </c>
+      <c r="B37" t="n">
+        <v>36</v>
+      </c>
+      <c r="C37" t="inlineStr">
+        <is>
+          <t>https://zigship.com</t>
+        </is>
+      </c>
+      <c r="D37" t="inlineStr">
+        <is>
+          <t>GET</t>
+        </is>
+      </c>
+      <c r="E37" t="n">
+        <v>2000</v>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" t="n">
+        <v>37</v>
+      </c>
+      <c r="B38" t="n">
+        <v>37</v>
+      </c>
+      <c r="C38" t="inlineStr">
+        <is>
+          <t>https://oneworldimmigration.ca</t>
+        </is>
+      </c>
+      <c r="D38" t="inlineStr">
+        <is>
+          <t>GET</t>
+        </is>
+      </c>
+      <c r="E38" t="n">
+        <v>2000</v>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" t="n">
+        <v>38</v>
+      </c>
+      <c r="B39" t="n">
+        <v>38</v>
+      </c>
+      <c r="C39" t="inlineStr">
+        <is>
+          <t>https://airconditioner-furnace.ca</t>
+        </is>
+      </c>
+      <c r="D39" t="inlineStr">
+        <is>
+          <t>GET</t>
+        </is>
+      </c>
+      <c r="E39" t="n">
+        <v>2000</v>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" t="n">
+        <v>39</v>
+      </c>
+      <c r="B40" t="n">
+        <v>39</v>
+      </c>
+      <c r="C40" t="inlineStr">
+        <is>
+          <t>https://bed-bugs-treatments.com</t>
+        </is>
+      </c>
+      <c r="D40" t="inlineStr">
+        <is>
+          <t>GET</t>
+        </is>
+      </c>
+      <c r="E40" t="n">
+        <v>2000</v>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" t="n">
+        <v>40</v>
+      </c>
+      <c r="B41" t="n">
+        <v>40</v>
+      </c>
+      <c r="C41" t="inlineStr">
+        <is>
+          <t>https://sultanxpress.ca</t>
+        </is>
+      </c>
+      <c r="D41" t="inlineStr">
+        <is>
+          <t>GET</t>
+        </is>
+      </c>
+      <c r="E41" t="n">
+        <v>2000</v>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" t="n">
+        <v>41</v>
+      </c>
+      <c r="B42" t="n">
+        <v>41</v>
+      </c>
+      <c r="C42" t="inlineStr">
+        <is>
+          <t>https://wildlifepro.ca</t>
+        </is>
+      </c>
+      <c r="D42" t="inlineStr">
+        <is>
+          <t>GET</t>
+        </is>
+      </c>
+      <c r="E42" t="n">
+        <v>2000</v>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" t="n">
+        <v>42</v>
+      </c>
+      <c r="B43" t="n">
+        <v>42</v>
+      </c>
+      <c r="C43" t="inlineStr">
+        <is>
+          <t>https://reboundproducts.com</t>
+        </is>
+      </c>
+      <c r="D43" t="inlineStr">
+        <is>
+          <t>GET</t>
+        </is>
+      </c>
+      <c r="E43" t="n">
         <v>2000</v>
       </c>
     </row>
@@ -678,7 +1915,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G2"/>
+  <dimension ref="A1:G1"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -718,37 +1955,6 @@
         </is>
       </c>
     </row>
-    <row r="2">
-      <c r="A2" t="inlineStr">
-        <is>
-          <t>GH_WEBGL_1</t>
-        </is>
-      </c>
-      <c r="B2" t="n">
-        <v>1</v>
-      </c>
-      <c r="C2" t="n">
-        <v>3</v>
-      </c>
-      <c r="D2" t="n">
-        <v>3</v>
-      </c>
-      <c r="E2" t="inlineStr">
-        <is>
-          <t>contains</t>
-        </is>
-      </c>
-      <c r="F2" t="inlineStr">
-        <is>
-          <t>GPU stall due to ReadPixels</t>
-        </is>
-      </c>
-      <c r="G2" t="inlineStr">
-        <is>
-          <t>Ignore GitHub WebGL GPU stall warning for testing</t>
-        </is>
-      </c>
-    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Update sites config: disable site ID 10
</commit_message>
<xml_diff>
--- a/data/sites.xlsx
+++ b/data/sites.xlsx
@@ -305,7 +305,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" mc:Ignorable="x14ac">
   <numFmts count="0"/>
-  <fonts count="3" x14ac:knownFonts="1">
+  <fonts count="4" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -316,6 +316,12 @@
     <font>
       <sz val="11"/>
       <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color rgb="FF000000"/>
       <name val="Calibri"/>
       <family val="2"/>
     </font>
@@ -362,13 +368,13 @@
     <xf xfId="0" numFmtId="0" borderId="0" fontId="0" fillId="0" applyAlignment="1">
       <alignment horizontal="general"/>
     </xf>
-    <xf xfId="0" numFmtId="3" applyNumberFormat="1" borderId="0" fontId="0" fillId="0" applyAlignment="1">
-      <alignment horizontal="right"/>
-    </xf>
     <xf xfId="0" numFmtId="3" applyNumberFormat="1" borderId="1" applyBorder="1" fontId="1" applyFont="1" fillId="0" applyAlignment="1">
       <alignment horizontal="right"/>
     </xf>
-    <xf xfId="0" numFmtId="0" borderId="1" applyBorder="1" fontId="2" applyFont="1" fillId="0" applyAlignment="1">
+    <xf xfId="0" numFmtId="3" applyNumberFormat="1" borderId="1" applyBorder="1" fontId="2" applyFont="1" fillId="0" applyAlignment="1">
+      <alignment horizontal="right"/>
+    </xf>
+    <xf xfId="0" numFmtId="0" borderId="1" applyBorder="1" fontId="3" applyFont="1" fillId="0" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
     <xf xfId="0" numFmtId="3" applyNumberFormat="1" borderId="0" fontId="0" fillId="0" applyAlignment="1">
@@ -695,7 +701,7 @@
         <v>1</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="2" customHeight="1" ht="18.75">
+    <row x14ac:dyDescent="0.25" r="2" customHeight="1" ht="19.5">
       <c r="A2" s="4">
         <v>1</v>
       </c>
@@ -706,7 +712,7 @@
         <v>1</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="3" customHeight="1" ht="18.75">
+    <row x14ac:dyDescent="0.25" r="3" customHeight="1" ht="19.5">
       <c r="A3" s="4">
         <v>2</v>
       </c>
@@ -717,7 +723,7 @@
         <v>1</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="4" customHeight="1" ht="18.75">
+    <row x14ac:dyDescent="0.25" r="4" customHeight="1" ht="19.5">
       <c r="A4" s="4">
         <v>3</v>
       </c>
@@ -728,7 +734,7 @@
         <v>1</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="5" customHeight="1" ht="18.75">
+    <row x14ac:dyDescent="0.25" r="5" customHeight="1" ht="19.5">
       <c r="A5" s="4">
         <v>4</v>
       </c>
@@ -739,7 +745,7 @@
         <v>1</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="6" customHeight="1" ht="18.75">
+    <row x14ac:dyDescent="0.25" r="6" customHeight="1" ht="19.5">
       <c r="A6" s="4">
         <v>5</v>
       </c>
@@ -750,7 +756,7 @@
         <v>1</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="7" customHeight="1" ht="18.75">
+    <row x14ac:dyDescent="0.25" r="7" customHeight="1" ht="19.5">
       <c r="A7" s="4">
         <v>6</v>
       </c>
@@ -761,7 +767,7 @@
         <v>1</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="8" customHeight="1" ht="18.75">
+    <row x14ac:dyDescent="0.25" r="8" customHeight="1" ht="19.5">
       <c r="A8" s="4">
         <v>7</v>
       </c>
@@ -772,7 +778,7 @@
         <v>1</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="9" customHeight="1" ht="18.75">
+    <row x14ac:dyDescent="0.25" r="9" customHeight="1" ht="19.5">
       <c r="A9" s="4">
         <v>8</v>
       </c>
@@ -783,7 +789,7 @@
         <v>1</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="10" customHeight="1" ht="18.75">
+    <row x14ac:dyDescent="0.25" r="10" customHeight="1" ht="19.5">
       <c r="A10" s="4">
         <v>9</v>
       </c>
@@ -794,7 +800,7 @@
         <v>1</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="11" customHeight="1" ht="18.75">
+    <row x14ac:dyDescent="0.25" r="11" customHeight="1" ht="19.5">
       <c r="A11" s="4">
         <v>10</v>
       </c>
@@ -802,10 +808,10 @@
         <v>62</v>
       </c>
       <c r="C11" s="4">
-        <v>1</v>
-      </c>
-    </row>
-    <row x14ac:dyDescent="0.25" r="12" customHeight="1" ht="18.75">
+        <v>0</v>
+      </c>
+    </row>
+    <row x14ac:dyDescent="0.25" r="12" customHeight="1" ht="19.5">
       <c r="A12" s="4">
         <v>11</v>
       </c>
@@ -816,7 +822,7 @@
         <v>1</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="13" customHeight="1" ht="18.75">
+    <row x14ac:dyDescent="0.25" r="13" customHeight="1" ht="19.5">
       <c r="A13" s="4">
         <v>12</v>
       </c>
@@ -827,7 +833,7 @@
         <v>1</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="14" customHeight="1" ht="18.75">
+    <row x14ac:dyDescent="0.25" r="14" customHeight="1" ht="19.5">
       <c r="A14" s="4">
         <v>13</v>
       </c>
@@ -838,7 +844,7 @@
         <v>1</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="15" customHeight="1" ht="18.75">
+    <row x14ac:dyDescent="0.25" r="15" customHeight="1" ht="19.5">
       <c r="A15" s="4">
         <v>14</v>
       </c>
@@ -849,7 +855,7 @@
         <v>1</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="16" customHeight="1" ht="18.75">
+    <row x14ac:dyDescent="0.25" r="16" customHeight="1" ht="19.5">
       <c r="A16" s="4">
         <v>15</v>
       </c>
@@ -860,7 +866,7 @@
         <v>1</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="17" customHeight="1" ht="18.75">
+    <row x14ac:dyDescent="0.25" r="17" customHeight="1" ht="19.5">
       <c r="A17" s="4">
         <v>16</v>
       </c>

</xml_diff>

<commit_message>
Update sites config: disable officecleninggta endpoint
</commit_message>
<xml_diff>
--- a/data/sites.xlsx
+++ b/data/sites.xlsx
@@ -305,19 +305,13 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" mc:Ignorable="x14ac">
   <numFmts count="0"/>
-  <fonts count="4" x14ac:knownFonts="1">
+  <fonts count="3" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
       <name val="Calibri"/>
       <family val="2"/>
       <scheme val="minor"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <color theme="1"/>
-      <name val="Calibri"/>
-      <family val="2"/>
     </font>
     <font>
       <sz val="11"/>
@@ -360,7 +354,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="7">
+  <cellXfs count="6">
     <xf xfId="0" numFmtId="0" borderId="0" fontId="0" fillId="0"/>
     <xf xfId="0" numFmtId="0" borderId="0" fontId="0" fillId="0" applyAlignment="1">
       <alignment horizontal="general"/>
@@ -371,10 +365,7 @@
     <xf xfId="0" numFmtId="3" applyNumberFormat="1" borderId="1" applyBorder="1" fontId="1" applyFont="1" fillId="0" applyAlignment="1">
       <alignment horizontal="right"/>
     </xf>
-    <xf xfId="0" numFmtId="3" applyNumberFormat="1" borderId="1" applyBorder="1" fontId="2" applyFont="1" fillId="0" applyAlignment="1">
-      <alignment horizontal="right"/>
-    </xf>
-    <xf xfId="0" numFmtId="0" borderId="1" applyBorder="1" fontId="3" applyFont="1" fillId="0" applyAlignment="1">
+    <xf xfId="0" numFmtId="0" borderId="1" applyBorder="1" fontId="2" applyFont="1" fillId="0" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
     <xf xfId="0" numFmtId="3" applyNumberFormat="1" borderId="0" fontId="0" fillId="0" applyAlignment="1">
@@ -685,12 +676,12 @@
   <dimension ref="A1:C43"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" style="6" width="13.576428571428572" customWidth="1" bestFit="1"/>
+    <col min="1" max="1" style="5" width="13.576428571428572" customWidth="1" bestFit="1"/>
     <col min="2" max="2" style="2" width="24.719285714285714" customWidth="1" bestFit="1"/>
-    <col min="3" max="3" style="6" width="13.576428571428572" customWidth="1" bestFit="1"/>
+    <col min="3" max="3" style="5" width="13.576428571428572" customWidth="1" bestFit="1"/>
   </cols>
   <sheetData>
-    <row x14ac:dyDescent="0.25" r="1" customHeight="1" ht="18.75">
+    <row x14ac:dyDescent="0.25" r="1" customHeight="1" ht="19.5">
       <c r="A1" s="3" t="s">
         <v>2</v>
       </c>
@@ -702,464 +693,464 @@
       </c>
     </row>
     <row x14ac:dyDescent="0.25" r="2" customHeight="1" ht="19.5">
-      <c r="A2" s="4">
+      <c r="A2" s="3">
         <v>1</v>
       </c>
       <c r="B2" s="1" t="s">
         <v>53</v>
       </c>
-      <c r="C2" s="4">
+      <c r="C2" s="3">
         <v>1</v>
       </c>
     </row>
     <row x14ac:dyDescent="0.25" r="3" customHeight="1" ht="19.5">
-      <c r="A3" s="4">
+      <c r="A3" s="3">
         <v>2</v>
       </c>
       <c r="B3" s="1" t="s">
         <v>54</v>
       </c>
-      <c r="C3" s="4">
+      <c r="C3" s="3">
         <v>1</v>
       </c>
     </row>
     <row x14ac:dyDescent="0.25" r="4" customHeight="1" ht="19.5">
-      <c r="A4" s="4">
+      <c r="A4" s="3">
         <v>3</v>
       </c>
       <c r="B4" s="1" t="s">
         <v>55</v>
       </c>
-      <c r="C4" s="4">
+      <c r="C4" s="3">
         <v>1</v>
       </c>
     </row>
     <row x14ac:dyDescent="0.25" r="5" customHeight="1" ht="19.5">
-      <c r="A5" s="4">
+      <c r="A5" s="3">
         <v>4</v>
       </c>
       <c r="B5" s="1" t="s">
         <v>56</v>
       </c>
-      <c r="C5" s="4">
+      <c r="C5" s="3">
         <v>1</v>
       </c>
     </row>
     <row x14ac:dyDescent="0.25" r="6" customHeight="1" ht="19.5">
-      <c r="A6" s="4">
+      <c r="A6" s="3">
         <v>5</v>
       </c>
       <c r="B6" s="1" t="s">
         <v>57</v>
       </c>
-      <c r="C6" s="4">
+      <c r="C6" s="3">
         <v>1</v>
       </c>
     </row>
     <row x14ac:dyDescent="0.25" r="7" customHeight="1" ht="19.5">
-      <c r="A7" s="4">
+      <c r="A7" s="3">
         <v>6</v>
       </c>
       <c r="B7" s="1" t="s">
         <v>58</v>
       </c>
-      <c r="C7" s="4">
+      <c r="C7" s="3">
         <v>1</v>
       </c>
     </row>
     <row x14ac:dyDescent="0.25" r="8" customHeight="1" ht="19.5">
-      <c r="A8" s="4">
+      <c r="A8" s="3">
         <v>7</v>
       </c>
       <c r="B8" s="1" t="s">
         <v>59</v>
       </c>
-      <c r="C8" s="4">
+      <c r="C8" s="3">
         <v>1</v>
       </c>
     </row>
     <row x14ac:dyDescent="0.25" r="9" customHeight="1" ht="19.5">
-      <c r="A9" s="4">
+      <c r="A9" s="3">
         <v>8</v>
       </c>
       <c r="B9" s="1" t="s">
         <v>60</v>
       </c>
-      <c r="C9" s="4">
+      <c r="C9" s="3">
         <v>1</v>
       </c>
     </row>
     <row x14ac:dyDescent="0.25" r="10" customHeight="1" ht="19.5">
-      <c r="A10" s="4">
+      <c r="A10" s="3">
         <v>9</v>
       </c>
       <c r="B10" s="1" t="s">
         <v>61</v>
       </c>
-      <c r="C10" s="4">
+      <c r="C10" s="3">
         <v>1</v>
       </c>
     </row>
     <row x14ac:dyDescent="0.25" r="11" customHeight="1" ht="19.5">
-      <c r="A11" s="4">
+      <c r="A11" s="3">
         <v>10</v>
       </c>
       <c r="B11" s="1" t="s">
         <v>62</v>
       </c>
-      <c r="C11" s="4">
+      <c r="C11" s="3">
         <v>0</v>
       </c>
     </row>
     <row x14ac:dyDescent="0.25" r="12" customHeight="1" ht="19.5">
-      <c r="A12" s="4">
+      <c r="A12" s="3">
         <v>11</v>
       </c>
       <c r="B12" s="1" t="s">
         <v>63</v>
       </c>
-      <c r="C12" s="4">
+      <c r="C12" s="3">
         <v>1</v>
       </c>
     </row>
     <row x14ac:dyDescent="0.25" r="13" customHeight="1" ht="19.5">
-      <c r="A13" s="4">
+      <c r="A13" s="3">
         <v>12</v>
       </c>
       <c r="B13" s="1" t="s">
         <v>64</v>
       </c>
-      <c r="C13" s="4">
+      <c r="C13" s="3">
         <v>1</v>
       </c>
     </row>
     <row x14ac:dyDescent="0.25" r="14" customHeight="1" ht="19.5">
-      <c r="A14" s="4">
+      <c r="A14" s="3">
         <v>13</v>
       </c>
       <c r="B14" s="1" t="s">
         <v>65</v>
       </c>
-      <c r="C14" s="4">
+      <c r="C14" s="3">
         <v>1</v>
       </c>
     </row>
     <row x14ac:dyDescent="0.25" r="15" customHeight="1" ht="19.5">
-      <c r="A15" s="4">
+      <c r="A15" s="3">
         <v>14</v>
       </c>
       <c r="B15" s="1" t="s">
         <v>66</v>
       </c>
-      <c r="C15" s="4">
+      <c r="C15" s="3">
         <v>1</v>
       </c>
     </row>
     <row x14ac:dyDescent="0.25" r="16" customHeight="1" ht="19.5">
-      <c r="A16" s="4">
+      <c r="A16" s="3">
         <v>15</v>
       </c>
       <c r="B16" s="1" t="s">
         <v>67</v>
       </c>
-      <c r="C16" s="4">
+      <c r="C16" s="3">
         <v>1</v>
       </c>
     </row>
     <row x14ac:dyDescent="0.25" r="17" customHeight="1" ht="19.5">
-      <c r="A17" s="4">
+      <c r="A17" s="3">
         <v>16</v>
       </c>
       <c r="B17" s="1" t="s">
         <v>68</v>
       </c>
-      <c r="C17" s="4">
+      <c r="C17" s="3">
         <v>1</v>
       </c>
     </row>
     <row x14ac:dyDescent="0.25" r="18" customHeight="1" ht="18.75">
-      <c r="A18" s="4">
+      <c r="A18" s="3">
         <v>17</v>
       </c>
       <c r="B18" s="1" t="s">
         <v>69</v>
       </c>
-      <c r="C18" s="4">
+      <c r="C18" s="3">
         <v>1</v>
       </c>
     </row>
     <row x14ac:dyDescent="0.25" r="19" customHeight="1" ht="18.75">
-      <c r="A19" s="4">
+      <c r="A19" s="3">
         <v>18</v>
       </c>
       <c r="B19" s="1" t="s">
         <v>70</v>
       </c>
-      <c r="C19" s="4">
+      <c r="C19" s="3">
         <v>1</v>
       </c>
     </row>
     <row x14ac:dyDescent="0.25" r="20" customHeight="1" ht="18.75">
-      <c r="A20" s="4">
+      <c r="A20" s="3">
         <v>19</v>
       </c>
       <c r="B20" s="1" t="s">
         <v>71</v>
       </c>
-      <c r="C20" s="4">
+      <c r="C20" s="3">
         <v>1</v>
       </c>
     </row>
     <row x14ac:dyDescent="0.25" r="21" customHeight="1" ht="18.75">
-      <c r="A21" s="4">
+      <c r="A21" s="3">
         <v>20</v>
       </c>
       <c r="B21" s="1" t="s">
         <v>72</v>
       </c>
-      <c r="C21" s="4">
+      <c r="C21" s="3">
         <v>1</v>
       </c>
     </row>
     <row x14ac:dyDescent="0.25" r="22" customHeight="1" ht="18.75">
-      <c r="A22" s="4">
+      <c r="A22" s="3">
         <v>21</v>
       </c>
       <c r="B22" s="1" t="s">
         <v>73</v>
       </c>
-      <c r="C22" s="4">
+      <c r="C22" s="3">
         <v>1</v>
       </c>
     </row>
     <row x14ac:dyDescent="0.25" r="23" customHeight="1" ht="18.75">
-      <c r="A23" s="4">
+      <c r="A23" s="3">
         <v>22</v>
       </c>
       <c r="B23" s="1" t="s">
         <v>74</v>
       </c>
-      <c r="C23" s="4">
+      <c r="C23" s="3">
         <v>1</v>
       </c>
     </row>
     <row x14ac:dyDescent="0.25" r="24" customHeight="1" ht="18.75">
-      <c r="A24" s="4">
+      <c r="A24" s="3">
         <v>23</v>
       </c>
       <c r="B24" s="1" t="s">
         <v>75</v>
       </c>
-      <c r="C24" s="4">
+      <c r="C24" s="3">
         <v>1</v>
       </c>
     </row>
     <row x14ac:dyDescent="0.25" r="25" customHeight="1" ht="18.75">
-      <c r="A25" s="4">
+      <c r="A25" s="3">
         <v>24</v>
       </c>
       <c r="B25" s="1" t="s">
         <v>76</v>
       </c>
-      <c r="C25" s="4">
+      <c r="C25" s="3">
         <v>1</v>
       </c>
     </row>
     <row x14ac:dyDescent="0.25" r="26" customHeight="1" ht="18.75">
-      <c r="A26" s="4">
+      <c r="A26" s="3">
         <v>25</v>
       </c>
       <c r="B26" s="1" t="s">
         <v>77</v>
       </c>
-      <c r="C26" s="4">
+      <c r="C26" s="3">
         <v>1</v>
       </c>
     </row>
     <row x14ac:dyDescent="0.25" r="27" customHeight="1" ht="18.75">
-      <c r="A27" s="4">
+      <c r="A27" s="3">
         <v>26</v>
       </c>
       <c r="B27" s="1" t="s">
         <v>78</v>
       </c>
-      <c r="C27" s="4">
-        <v>1</v>
+      <c r="C27" s="3">
+        <v>0</v>
       </c>
     </row>
     <row x14ac:dyDescent="0.25" r="28" customHeight="1" ht="18.75">
-      <c r="A28" s="4">
+      <c r="A28" s="3">
         <v>27</v>
       </c>
       <c r="B28" s="1" t="s">
         <v>79</v>
       </c>
-      <c r="C28" s="4">
+      <c r="C28" s="3">
         <v>1</v>
       </c>
     </row>
     <row x14ac:dyDescent="0.25" r="29" customHeight="1" ht="18.75">
-      <c r="A29" s="4">
+      <c r="A29" s="3">
         <v>28</v>
       </c>
       <c r="B29" s="1" t="s">
         <v>80</v>
       </c>
-      <c r="C29" s="4">
+      <c r="C29" s="3">
         <v>1</v>
       </c>
     </row>
     <row x14ac:dyDescent="0.25" r="30" customHeight="1" ht="18.75">
-      <c r="A30" s="4">
+      <c r="A30" s="3">
         <v>29</v>
       </c>
       <c r="B30" s="1" t="s">
         <v>81</v>
       </c>
-      <c r="C30" s="4">
+      <c r="C30" s="3">
         <v>1</v>
       </c>
     </row>
     <row x14ac:dyDescent="0.25" r="31" customHeight="1" ht="18.75">
-      <c r="A31" s="4">
+      <c r="A31" s="3">
         <v>30</v>
       </c>
       <c r="B31" s="1" t="s">
         <v>82</v>
       </c>
-      <c r="C31" s="4">
+      <c r="C31" s="3">
         <v>1</v>
       </c>
     </row>
     <row x14ac:dyDescent="0.25" r="32" customHeight="1" ht="18.75">
-      <c r="A32" s="4">
+      <c r="A32" s="3">
         <v>31</v>
       </c>
       <c r="B32" s="1" t="s">
         <v>83</v>
       </c>
-      <c r="C32" s="4">
+      <c r="C32" s="3">
         <v>1</v>
       </c>
     </row>
     <row x14ac:dyDescent="0.25" r="33" customHeight="1" ht="18.75">
-      <c r="A33" s="4">
+      <c r="A33" s="3">
         <v>32</v>
       </c>
       <c r="B33" s="1" t="s">
         <v>84</v>
       </c>
-      <c r="C33" s="4">
+      <c r="C33" s="3">
         <v>1</v>
       </c>
     </row>
     <row x14ac:dyDescent="0.25" r="34" customHeight="1" ht="18.75">
-      <c r="A34" s="4">
+      <c r="A34" s="3">
         <v>33</v>
       </c>
       <c r="B34" s="1" t="s">
         <v>85</v>
       </c>
-      <c r="C34" s="4">
+      <c r="C34" s="3">
         <v>1</v>
       </c>
     </row>
     <row x14ac:dyDescent="0.25" r="35" customHeight="1" ht="18.75">
-      <c r="A35" s="4">
+      <c r="A35" s="3">
         <v>34</v>
       </c>
       <c r="B35" s="1" t="s">
         <v>86</v>
       </c>
-      <c r="C35" s="4">
+      <c r="C35" s="3">
         <v>0</v>
       </c>
     </row>
     <row x14ac:dyDescent="0.25" r="36" customHeight="1" ht="18.75">
-      <c r="A36" s="4">
+      <c r="A36" s="3">
         <v>35</v>
       </c>
       <c r="B36" s="1" t="s">
         <v>87</v>
       </c>
-      <c r="C36" s="4">
+      <c r="C36" s="3">
         <v>1</v>
       </c>
     </row>
     <row x14ac:dyDescent="0.25" r="37" customHeight="1" ht="18.75">
-      <c r="A37" s="4">
+      <c r="A37" s="3">
         <v>36</v>
       </c>
       <c r="B37" s="1" t="s">
         <v>88</v>
       </c>
-      <c r="C37" s="4">
+      <c r="C37" s="3">
         <v>1</v>
       </c>
     </row>
     <row x14ac:dyDescent="0.25" r="38" customHeight="1" ht="18.75">
-      <c r="A38" s="4">
+      <c r="A38" s="3">
         <v>37</v>
       </c>
       <c r="B38" s="1" t="s">
         <v>89</v>
       </c>
-      <c r="C38" s="4">
+      <c r="C38" s="3">
         <v>1</v>
       </c>
     </row>
     <row x14ac:dyDescent="0.25" r="39" customHeight="1" ht="18.75">
-      <c r="A39" s="4">
+      <c r="A39" s="3">
         <v>38</v>
       </c>
       <c r="B39" s="1" t="s">
         <v>90</v>
       </c>
-      <c r="C39" s="4">
+      <c r="C39" s="3">
         <v>1</v>
       </c>
     </row>
     <row x14ac:dyDescent="0.25" r="40" customHeight="1" ht="18.75">
-      <c r="A40" s="4">
+      <c r="A40" s="3">
         <v>39</v>
       </c>
       <c r="B40" s="1" t="s">
         <v>91</v>
       </c>
-      <c r="C40" s="4">
+      <c r="C40" s="3">
         <v>1</v>
       </c>
     </row>
     <row x14ac:dyDescent="0.25" r="41" customHeight="1" ht="18.75">
-      <c r="A41" s="4">
+      <c r="A41" s="3">
         <v>40</v>
       </c>
       <c r="B41" s="1" t="s">
         <v>92</v>
       </c>
-      <c r="C41" s="4">
+      <c r="C41" s="3">
         <v>1</v>
       </c>
     </row>
     <row x14ac:dyDescent="0.25" r="42" customHeight="1" ht="18.75">
-      <c r="A42" s="4">
+      <c r="A42" s="3">
         <v>41</v>
       </c>
       <c r="B42" s="1" t="s">
         <v>86</v>
       </c>
-      <c r="C42" s="4">
+      <c r="C42" s="3">
         <v>1</v>
       </c>
     </row>
     <row x14ac:dyDescent="0.25" r="43" customHeight="1" ht="18.75">
-      <c r="A43" s="4">
+      <c r="A43" s="3">
         <v>42</v>
       </c>
       <c r="B43" s="1" t="s">
         <v>93</v>
       </c>
-      <c r="C43" s="4">
+      <c r="C43" s="3">
         <v>1</v>
       </c>
     </row>
@@ -1176,11 +1167,11 @@
   <dimension ref="A1:E43"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" style="6" width="13.576428571428572" customWidth="1" bestFit="1"/>
-    <col min="2" max="2" style="6" width="13.576428571428572" customWidth="1" bestFit="1"/>
+    <col min="1" max="1" style="5" width="13.576428571428572" customWidth="1" bestFit="1"/>
+    <col min="2" max="2" style="5" width="13.576428571428572" customWidth="1" bestFit="1"/>
     <col min="3" max="3" style="2" width="47.14785714285715" customWidth="1" bestFit="1"/>
     <col min="4" max="4" style="2" width="13.576428571428572" customWidth="1" bestFit="1"/>
-    <col min="5" max="5" style="6" width="13.576428571428572" customWidth="1" bestFit="1"/>
+    <col min="5" max="5" style="5" width="13.576428571428572" customWidth="1" bestFit="1"/>
   </cols>
   <sheetData>
     <row x14ac:dyDescent="0.25" r="1" customHeight="1" ht="18.75">
@@ -1201,10 +1192,10 @@
       </c>
     </row>
     <row x14ac:dyDescent="0.25" r="2" customHeight="1" ht="18.75">
-      <c r="A2" s="4">
-        <v>1</v>
-      </c>
-      <c r="B2" s="4">
+      <c r="A2" s="3">
+        <v>1</v>
+      </c>
+      <c r="B2" s="3">
         <v>1</v>
       </c>
       <c r="C2" s="1" t="s">
@@ -1213,15 +1204,15 @@
       <c r="D2" s="1" t="s">
         <v>11</v>
       </c>
-      <c r="E2" s="4">
+      <c r="E2" s="3">
         <v>2000</v>
       </c>
     </row>
     <row x14ac:dyDescent="0.25" r="3" customHeight="1" ht="18.75">
-      <c r="A3" s="4">
+      <c r="A3" s="3">
         <v>2</v>
       </c>
-      <c r="B3" s="4">
+      <c r="B3" s="3">
         <v>2</v>
       </c>
       <c r="C3" s="1" t="s">
@@ -1230,15 +1221,15 @@
       <c r="D3" s="1" t="s">
         <v>11</v>
       </c>
-      <c r="E3" s="4">
+      <c r="E3" s="3">
         <v>2000</v>
       </c>
     </row>
     <row x14ac:dyDescent="0.25" r="4" customHeight="1" ht="18.75">
-      <c r="A4" s="4">
+      <c r="A4" s="3">
         <v>3</v>
       </c>
-      <c r="B4" s="4">
+      <c r="B4" s="3">
         <v>3</v>
       </c>
       <c r="C4" s="1" t="s">
@@ -1247,15 +1238,15 @@
       <c r="D4" s="1" t="s">
         <v>11</v>
       </c>
-      <c r="E4" s="4">
+      <c r="E4" s="3">
         <v>2000</v>
       </c>
     </row>
     <row x14ac:dyDescent="0.25" r="5" customHeight="1" ht="18.75">
-      <c r="A5" s="4">
+      <c r="A5" s="3">
         <v>4</v>
       </c>
-      <c r="B5" s="4">
+      <c r="B5" s="3">
         <v>4</v>
       </c>
       <c r="C5" s="1" t="s">
@@ -1264,15 +1255,15 @@
       <c r="D5" s="1" t="s">
         <v>11</v>
       </c>
-      <c r="E5" s="4">
+      <c r="E5" s="3">
         <v>2000</v>
       </c>
     </row>
     <row x14ac:dyDescent="0.25" r="6" customHeight="1" ht="18.75">
-      <c r="A6" s="4">
+      <c r="A6" s="3">
         <v>5</v>
       </c>
-      <c r="B6" s="4">
+      <c r="B6" s="3">
         <v>5</v>
       </c>
       <c r="C6" s="1" t="s">
@@ -1281,15 +1272,15 @@
       <c r="D6" s="1" t="s">
         <v>11</v>
       </c>
-      <c r="E6" s="4">
+      <c r="E6" s="3">
         <v>2000</v>
       </c>
     </row>
     <row x14ac:dyDescent="0.25" r="7" customHeight="1" ht="18.75">
-      <c r="A7" s="4">
+      <c r="A7" s="3">
         <v>6</v>
       </c>
-      <c r="B7" s="4">
+      <c r="B7" s="3">
         <v>6</v>
       </c>
       <c r="C7" s="1" t="s">
@@ -1298,15 +1289,15 @@
       <c r="D7" s="1" t="s">
         <v>11</v>
       </c>
-      <c r="E7" s="4">
+      <c r="E7" s="3">
         <v>2000</v>
       </c>
     </row>
     <row x14ac:dyDescent="0.25" r="8" customHeight="1" ht="18.75">
-      <c r="A8" s="4">
+      <c r="A8" s="3">
         <v>7</v>
       </c>
-      <c r="B8" s="4">
+      <c r="B8" s="3">
         <v>7</v>
       </c>
       <c r="C8" s="1" t="s">
@@ -1315,15 +1306,15 @@
       <c r="D8" s="1" t="s">
         <v>11</v>
       </c>
-      <c r="E8" s="4">
+      <c r="E8" s="3">
         <v>2000</v>
       </c>
     </row>
     <row x14ac:dyDescent="0.25" r="9" customHeight="1" ht="18.75">
-      <c r="A9" s="4">
+      <c r="A9" s="3">
         <v>8</v>
       </c>
-      <c r="B9" s="4">
+      <c r="B9" s="3">
         <v>8</v>
       </c>
       <c r="C9" s="1" t="s">
@@ -1332,15 +1323,15 @@
       <c r="D9" s="1" t="s">
         <v>11</v>
       </c>
-      <c r="E9" s="4">
+      <c r="E9" s="3">
         <v>2000</v>
       </c>
     </row>
     <row x14ac:dyDescent="0.25" r="10" customHeight="1" ht="18.75">
-      <c r="A10" s="4">
+      <c r="A10" s="3">
         <v>9</v>
       </c>
-      <c r="B10" s="4">
+      <c r="B10" s="3">
         <v>9</v>
       </c>
       <c r="C10" s="1" t="s">
@@ -1349,15 +1340,15 @@
       <c r="D10" s="1" t="s">
         <v>11</v>
       </c>
-      <c r="E10" s="4">
+      <c r="E10" s="3">
         <v>2000</v>
       </c>
     </row>
     <row x14ac:dyDescent="0.25" r="11" customHeight="1" ht="18.75">
-      <c r="A11" s="4">
+      <c r="A11" s="3">
         <v>10</v>
       </c>
-      <c r="B11" s="4">
+      <c r="B11" s="3">
         <v>10</v>
       </c>
       <c r="C11" s="1" t="s">
@@ -1366,15 +1357,15 @@
       <c r="D11" s="1" t="s">
         <v>11</v>
       </c>
-      <c r="E11" s="4">
+      <c r="E11" s="3">
         <v>2000</v>
       </c>
     </row>
     <row x14ac:dyDescent="0.25" r="12" customHeight="1" ht="18.75">
-      <c r="A12" s="4">
-        <v>11</v>
-      </c>
-      <c r="B12" s="4">
+      <c r="A12" s="3">
+        <v>11</v>
+      </c>
+      <c r="B12" s="3">
         <v>11</v>
       </c>
       <c r="C12" s="1" t="s">
@@ -1383,15 +1374,15 @@
       <c r="D12" s="1" t="s">
         <v>11</v>
       </c>
-      <c r="E12" s="4">
+      <c r="E12" s="3">
         <v>2000</v>
       </c>
     </row>
     <row x14ac:dyDescent="0.25" r="13" customHeight="1" ht="18.75">
-      <c r="A13" s="4">
+      <c r="A13" s="3">
         <v>12</v>
       </c>
-      <c r="B13" s="4">
+      <c r="B13" s="3">
         <v>12</v>
       </c>
       <c r="C13" s="1" t="s">
@@ -1400,15 +1391,15 @@
       <c r="D13" s="1" t="s">
         <v>11</v>
       </c>
-      <c r="E13" s="4">
+      <c r="E13" s="3">
         <v>2000</v>
       </c>
     </row>
     <row x14ac:dyDescent="0.25" r="14" customHeight="1" ht="18.75">
-      <c r="A14" s="4">
+      <c r="A14" s="3">
         <v>13</v>
       </c>
-      <c r="B14" s="4">
+      <c r="B14" s="3">
         <v>13</v>
       </c>
       <c r="C14" s="1" t="s">
@@ -1417,15 +1408,15 @@
       <c r="D14" s="1" t="s">
         <v>11</v>
       </c>
-      <c r="E14" s="4">
+      <c r="E14" s="3">
         <v>2000</v>
       </c>
     </row>
     <row x14ac:dyDescent="0.25" r="15" customHeight="1" ht="18.75">
-      <c r="A15" s="4">
+      <c r="A15" s="3">
         <v>14</v>
       </c>
-      <c r="B15" s="4">
+      <c r="B15" s="3">
         <v>14</v>
       </c>
       <c r="C15" s="1" t="s">
@@ -1434,15 +1425,15 @@
       <c r="D15" s="1" t="s">
         <v>11</v>
       </c>
-      <c r="E15" s="4">
+      <c r="E15" s="3">
         <v>2000</v>
       </c>
     </row>
     <row x14ac:dyDescent="0.25" r="16" customHeight="1" ht="18.75">
-      <c r="A16" s="4">
+      <c r="A16" s="3">
         <v>15</v>
       </c>
-      <c r="B16" s="4">
+      <c r="B16" s="3">
         <v>15</v>
       </c>
       <c r="C16" s="1" t="s">
@@ -1451,15 +1442,15 @@
       <c r="D16" s="1" t="s">
         <v>11</v>
       </c>
-      <c r="E16" s="4">
+      <c r="E16" s="3">
         <v>2000</v>
       </c>
     </row>
     <row x14ac:dyDescent="0.25" r="17" customHeight="1" ht="18.75">
-      <c r="A17" s="4">
+      <c r="A17" s="3">
         <v>16</v>
       </c>
-      <c r="B17" s="4">
+      <c r="B17" s="3">
         <v>16</v>
       </c>
       <c r="C17" s="1" t="s">
@@ -1468,15 +1459,15 @@
       <c r="D17" s="1" t="s">
         <v>11</v>
       </c>
-      <c r="E17" s="4">
+      <c r="E17" s="3">
         <v>2000</v>
       </c>
     </row>
     <row x14ac:dyDescent="0.25" r="18" customHeight="1" ht="18.75">
-      <c r="A18" s="4">
+      <c r="A18" s="3">
         <v>17</v>
       </c>
-      <c r="B18" s="4">
+      <c r="B18" s="3">
         <v>17</v>
       </c>
       <c r="C18" s="1" t="s">
@@ -1485,15 +1476,15 @@
       <c r="D18" s="1" t="s">
         <v>11</v>
       </c>
-      <c r="E18" s="4">
+      <c r="E18" s="3">
         <v>2000</v>
       </c>
     </row>
     <row x14ac:dyDescent="0.25" r="19" customHeight="1" ht="18.75">
-      <c r="A19" s="4">
+      <c r="A19" s="3">
         <v>18</v>
       </c>
-      <c r="B19" s="4">
+      <c r="B19" s="3">
         <v>18</v>
       </c>
       <c r="C19" s="1" t="s">
@@ -1502,15 +1493,15 @@
       <c r="D19" s="1" t="s">
         <v>11</v>
       </c>
-      <c r="E19" s="4">
+      <c r="E19" s="3">
         <v>2000</v>
       </c>
     </row>
     <row x14ac:dyDescent="0.25" r="20" customHeight="1" ht="18.75">
-      <c r="A20" s="4">
+      <c r="A20" s="3">
         <v>19</v>
       </c>
-      <c r="B20" s="4">
+      <c r="B20" s="3">
         <v>19</v>
       </c>
       <c r="C20" s="1" t="s">
@@ -1519,15 +1510,15 @@
       <c r="D20" s="1" t="s">
         <v>11</v>
       </c>
-      <c r="E20" s="4">
+      <c r="E20" s="3">
         <v>2000</v>
       </c>
     </row>
     <row x14ac:dyDescent="0.25" r="21" customHeight="1" ht="18.75">
-      <c r="A21" s="4">
+      <c r="A21" s="3">
         <v>20</v>
       </c>
-      <c r="B21" s="4">
+      <c r="B21" s="3">
         <v>20</v>
       </c>
       <c r="C21" s="1" t="s">
@@ -1536,15 +1527,15 @@
       <c r="D21" s="1" t="s">
         <v>11</v>
       </c>
-      <c r="E21" s="4">
+      <c r="E21" s="3">
         <v>2000</v>
       </c>
     </row>
     <row x14ac:dyDescent="0.25" r="22" customHeight="1" ht="18.75">
-      <c r="A22" s="4">
+      <c r="A22" s="3">
         <v>21</v>
       </c>
-      <c r="B22" s="4">
+      <c r="B22" s="3">
         <v>21</v>
       </c>
       <c r="C22" s="1" t="s">
@@ -1553,15 +1544,15 @@
       <c r="D22" s="1" t="s">
         <v>11</v>
       </c>
-      <c r="E22" s="4">
+      <c r="E22" s="3">
         <v>2000</v>
       </c>
     </row>
     <row x14ac:dyDescent="0.25" r="23" customHeight="1" ht="18.75">
-      <c r="A23" s="4">
+      <c r="A23" s="3">
         <v>22</v>
       </c>
-      <c r="B23" s="4">
+      <c r="B23" s="3">
         <v>22</v>
       </c>
       <c r="C23" s="1" t="s">
@@ -1570,15 +1561,15 @@
       <c r="D23" s="1" t="s">
         <v>11</v>
       </c>
-      <c r="E23" s="4">
+      <c r="E23" s="3">
         <v>2000</v>
       </c>
     </row>
     <row x14ac:dyDescent="0.25" r="24" customHeight="1" ht="18.75">
-      <c r="A24" s="4">
+      <c r="A24" s="3">
         <v>23</v>
       </c>
-      <c r="B24" s="4">
+      <c r="B24" s="3">
         <v>23</v>
       </c>
       <c r="C24" s="1" t="s">
@@ -1587,15 +1578,15 @@
       <c r="D24" s="1" t="s">
         <v>11</v>
       </c>
-      <c r="E24" s="4">
+      <c r="E24" s="3">
         <v>2000</v>
       </c>
     </row>
     <row x14ac:dyDescent="0.25" r="25" customHeight="1" ht="18.75">
-      <c r="A25" s="4">
+      <c r="A25" s="3">
         <v>24</v>
       </c>
-      <c r="B25" s="4">
+      <c r="B25" s="3">
         <v>24</v>
       </c>
       <c r="C25" s="1" t="s">
@@ -1604,15 +1595,15 @@
       <c r="D25" s="1" t="s">
         <v>11</v>
       </c>
-      <c r="E25" s="4">
+      <c r="E25" s="3">
         <v>2000</v>
       </c>
     </row>
     <row x14ac:dyDescent="0.25" r="26" customHeight="1" ht="18.75">
-      <c r="A26" s="4">
+      <c r="A26" s="3">
         <v>25</v>
       </c>
-      <c r="B26" s="4">
+      <c r="B26" s="3">
         <v>25</v>
       </c>
       <c r="C26" s="1" t="s">
@@ -1621,15 +1612,15 @@
       <c r="D26" s="1" t="s">
         <v>11</v>
       </c>
-      <c r="E26" s="4">
+      <c r="E26" s="3">
         <v>2000</v>
       </c>
     </row>
     <row x14ac:dyDescent="0.25" r="27" customHeight="1" ht="18.75">
-      <c r="A27" s="4">
+      <c r="A27" s="3">
         <v>26</v>
       </c>
-      <c r="B27" s="4">
+      <c r="B27" s="3">
         <v>26</v>
       </c>
       <c r="C27" s="1" t="s">
@@ -1638,15 +1629,15 @@
       <c r="D27" s="1" t="s">
         <v>11</v>
       </c>
-      <c r="E27" s="4">
+      <c r="E27" s="3">
         <v>2000</v>
       </c>
     </row>
     <row x14ac:dyDescent="0.25" r="28" customHeight="1" ht="18.75">
-      <c r="A28" s="4">
+      <c r="A28" s="3">
         <v>27</v>
       </c>
-      <c r="B28" s="4">
+      <c r="B28" s="3">
         <v>27</v>
       </c>
       <c r="C28" s="1" t="s">
@@ -1655,15 +1646,15 @@
       <c r="D28" s="1" t="s">
         <v>11</v>
       </c>
-      <c r="E28" s="4">
+      <c r="E28" s="3">
         <v>2000</v>
       </c>
     </row>
     <row x14ac:dyDescent="0.25" r="29" customHeight="1" ht="18.75">
-      <c r="A29" s="4">
+      <c r="A29" s="3">
         <v>28</v>
       </c>
-      <c r="B29" s="4">
+      <c r="B29" s="3">
         <v>28</v>
       </c>
       <c r="C29" s="1" t="s">
@@ -1672,15 +1663,15 @@
       <c r="D29" s="1" t="s">
         <v>11</v>
       </c>
-      <c r="E29" s="4">
+      <c r="E29" s="3">
         <v>2000</v>
       </c>
     </row>
     <row x14ac:dyDescent="0.25" r="30" customHeight="1" ht="18.75">
-      <c r="A30" s="4">
+      <c r="A30" s="3">
         <v>29</v>
       </c>
-      <c r="B30" s="4">
+      <c r="B30" s="3">
         <v>29</v>
       </c>
       <c r="C30" s="1" t="s">
@@ -1689,15 +1680,15 @@
       <c r="D30" s="1" t="s">
         <v>11</v>
       </c>
-      <c r="E30" s="4">
+      <c r="E30" s="3">
         <v>2000</v>
       </c>
     </row>
     <row x14ac:dyDescent="0.25" r="31" customHeight="1" ht="18.75">
-      <c r="A31" s="4">
+      <c r="A31" s="3">
         <v>30</v>
       </c>
-      <c r="B31" s="4">
+      <c r="B31" s="3">
         <v>30</v>
       </c>
       <c r="C31" s="1" t="s">
@@ -1706,15 +1697,15 @@
       <c r="D31" s="1" t="s">
         <v>11</v>
       </c>
-      <c r="E31" s="4">
+      <c r="E31" s="3">
         <v>2000</v>
       </c>
     </row>
     <row x14ac:dyDescent="0.25" r="32" customHeight="1" ht="18.75">
-      <c r="A32" s="4">
+      <c r="A32" s="3">
         <v>31</v>
       </c>
-      <c r="B32" s="4">
+      <c r="B32" s="3">
         <v>31</v>
       </c>
       <c r="C32" s="1" t="s">
@@ -1723,32 +1714,32 @@
       <c r="D32" s="1" t="s">
         <v>11</v>
       </c>
-      <c r="E32" s="4">
+      <c r="E32" s="3">
         <v>2000</v>
       </c>
     </row>
     <row x14ac:dyDescent="0.25" r="33" customHeight="1" ht="18.75">
-      <c r="A33" s="4">
+      <c r="A33" s="3">
         <v>32</v>
       </c>
-      <c r="B33" s="4">
+      <c r="B33" s="3">
         <v>32</v>
       </c>
-      <c r="C33" s="5" t="s">
+      <c r="C33" s="4" t="s">
         <v>42</v>
       </c>
       <c r="D33" s="1" t="s">
         <v>11</v>
       </c>
-      <c r="E33" s="4">
+      <c r="E33" s="3">
         <v>2000</v>
       </c>
     </row>
     <row x14ac:dyDescent="0.25" r="34" customHeight="1" ht="18.75">
-      <c r="A34" s="4">
+      <c r="A34" s="3">
         <v>33</v>
       </c>
-      <c r="B34" s="4">
+      <c r="B34" s="3">
         <v>33</v>
       </c>
       <c r="C34" s="1" t="s">
@@ -1757,32 +1748,32 @@
       <c r="D34" s="1" t="s">
         <v>11</v>
       </c>
-      <c r="E34" s="4">
+      <c r="E34" s="3">
         <v>2000</v>
       </c>
     </row>
     <row x14ac:dyDescent="0.25" r="35" customHeight="1" ht="18.75">
-      <c r="A35" s="4">
+      <c r="A35" s="3">
         <v>34</v>
       </c>
-      <c r="B35" s="4">
+      <c r="B35" s="3">
         <v>34</v>
       </c>
-      <c r="C35" s="5" t="s">
+      <c r="C35" s="4" t="s">
         <v>44</v>
       </c>
       <c r="D35" s="1" t="s">
         <v>11</v>
       </c>
-      <c r="E35" s="4">
+      <c r="E35" s="3">
         <v>2000</v>
       </c>
     </row>
     <row x14ac:dyDescent="0.25" r="36" customHeight="1" ht="18.75">
-      <c r="A36" s="4">
+      <c r="A36" s="3">
         <v>35</v>
       </c>
-      <c r="B36" s="4">
+      <c r="B36" s="3">
         <v>35</v>
       </c>
       <c r="C36" s="1" t="s">
@@ -1791,15 +1782,15 @@
       <c r="D36" s="1" t="s">
         <v>11</v>
       </c>
-      <c r="E36" s="4">
+      <c r="E36" s="3">
         <v>2000</v>
       </c>
     </row>
     <row x14ac:dyDescent="0.25" r="37" customHeight="1" ht="18.75">
-      <c r="A37" s="4">
+      <c r="A37" s="3">
         <v>36</v>
       </c>
-      <c r="B37" s="4">
+      <c r="B37" s="3">
         <v>36</v>
       </c>
       <c r="C37" s="1" t="s">
@@ -1808,15 +1799,15 @@
       <c r="D37" s="1" t="s">
         <v>11</v>
       </c>
-      <c r="E37" s="4">
+      <c r="E37" s="3">
         <v>2000</v>
       </c>
     </row>
     <row x14ac:dyDescent="0.25" r="38" customHeight="1" ht="18.75">
-      <c r="A38" s="4">
+      <c r="A38" s="3">
         <v>37</v>
       </c>
-      <c r="B38" s="4">
+      <c r="B38" s="3">
         <v>37</v>
       </c>
       <c r="C38" s="1" t="s">
@@ -1825,15 +1816,15 @@
       <c r="D38" s="1" t="s">
         <v>11</v>
       </c>
-      <c r="E38" s="4">
+      <c r="E38" s="3">
         <v>2000</v>
       </c>
     </row>
     <row x14ac:dyDescent="0.25" r="39" customHeight="1" ht="18.75">
-      <c r="A39" s="4">
+      <c r="A39" s="3">
         <v>38</v>
       </c>
-      <c r="B39" s="4">
+      <c r="B39" s="3">
         <v>38</v>
       </c>
       <c r="C39" s="1" t="s">
@@ -1842,15 +1833,15 @@
       <c r="D39" s="1" t="s">
         <v>11</v>
       </c>
-      <c r="E39" s="4">
+      <c r="E39" s="3">
         <v>2000</v>
       </c>
     </row>
     <row x14ac:dyDescent="0.25" r="40" customHeight="1" ht="18.75">
-      <c r="A40" s="4">
+      <c r="A40" s="3">
         <v>39</v>
       </c>
-      <c r="B40" s="4">
+      <c r="B40" s="3">
         <v>39</v>
       </c>
       <c r="C40" s="1" t="s">
@@ -1859,15 +1850,15 @@
       <c r="D40" s="1" t="s">
         <v>11</v>
       </c>
-      <c r="E40" s="4">
+      <c r="E40" s="3">
         <v>2000</v>
       </c>
     </row>
     <row x14ac:dyDescent="0.25" r="41" customHeight="1" ht="18.75">
-      <c r="A41" s="4">
+      <c r="A41" s="3">
         <v>40</v>
       </c>
-      <c r="B41" s="4">
+      <c r="B41" s="3">
         <v>40</v>
       </c>
       <c r="C41" s="1" t="s">
@@ -1876,32 +1867,32 @@
       <c r="D41" s="1" t="s">
         <v>11</v>
       </c>
-      <c r="E41" s="4">
+      <c r="E41" s="3">
         <v>2000</v>
       </c>
     </row>
     <row x14ac:dyDescent="0.25" r="42" customHeight="1" ht="18.75">
-      <c r="A42" s="4">
+      <c r="A42" s="3">
         <v>41</v>
       </c>
-      <c r="B42" s="4">
+      <c r="B42" s="3">
         <v>41</v>
       </c>
-      <c r="C42" s="5" t="s">
+      <c r="C42" s="4" t="s">
         <v>44</v>
       </c>
       <c r="D42" s="1" t="s">
         <v>11</v>
       </c>
-      <c r="E42" s="4">
+      <c r="E42" s="3">
         <v>2000</v>
       </c>
     </row>
     <row x14ac:dyDescent="0.25" r="43" customHeight="1" ht="18.75">
-      <c r="A43" s="4">
+      <c r="A43" s="3">
         <v>42</v>
       </c>
-      <c r="B43" s="4">
+      <c r="B43" s="3">
         <v>42</v>
       </c>
       <c r="C43" s="1" t="s">
@@ -1910,7 +1901,7 @@
       <c r="D43" s="1" t="s">
         <v>11</v>
       </c>
-      <c r="E43" s="4">
+      <c r="E43" s="3">
         <v>2000</v>
       </c>
     </row>

</xml_diff>